<commit_message>
add nissan leaf to BOM
</commit_message>
<xml_diff>
--- a/Documentation/BOM_Wireless_DBW.xlsx
+++ b/Documentation/BOM_Wireless_DBW.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -769,18 +769,46 @@
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="5" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Used Car Market</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Nissan Leaf (used, model year 2015–2018)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F12" s="4">
+        <f>D12*E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="F12" s="6">
-        <f>SUM(F2:F11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="F13" s="6">
+        <f>SUM(F2:F12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14"/>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>* OCI server uses Oracle Always Free Tier — no cost incurred.</t>
         </is>

</xml_diff>

<commit_message>
add user manual and design document; pep8 python files; update BOM
</commit_message>
<xml_diff>
--- a/Documentation/BOM_Wireless_DBW.xlsx
+++ b/Documentation/BOM_Wireless_DBW.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,8 +53,26 @@
       <color rgb="00595959"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00375623"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -64,6 +82,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -90,6 +113,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -455,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -464,6 +493,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -497,32 +527,42 @@
           <t>Total Cost</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="8" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>B08D5ZD528</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>Logitech G29 Driving Force Racing Wheel + Pedals</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="3" t="n">
+      <c r="D2" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="9" t="n">
         <v>249.99</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="9">
         <f>D2*E2</f>
         <v/>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>★ Purchased — budget item</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -814,9 +854,21 @@
         </is>
       </c>
     </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>★ Budget note: all components except the Logitech G29 were provided by the university or were already on hand. The team's out-of-pocket budget consisted solely of the G29 driving simulator ($249.99).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A14:F14"/>
+  <mergeCells count="2">
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A15:G15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix audit inaccuracies; simplify README; clean up BOM notes
- design_doc.tex: correct DAC baseline counts to match float32 truncation
  in firmware (steer 2473->2469, accel1 370->369, accel2 750->749,
  brake1 3417->3419; brake2 1509 unchanged)
- README.md: rewrite as concise reference — add repo URL, keep only
  System Overview, Hardware Requirements (component table), Software
  Requirements, Setup, and Running the System; fix seq=00001->seq=00000
- BOM: remove OCI footnote row, strip asterisk from OCI description,
  update budget note to reflect G29 as sole out-of-pocket purchase
  shared amongst capstone teams
- Recompile design_doc.pdf

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/BOM_Wireless_DBW.xlsx
+++ b/Documentation/BOM_Wireless_DBW.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -740,7 +740,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>OCI VM.Standard.E2.1.Micro Compute Instance (Always Free*)</t>
+          <t>OCI VM.Standard.E2.1.Micro Compute Instance (Always Free)</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -846,30 +846,17 @@
         <v/>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>* OCI server uses Oracle Always Free Tier — no cost incurred.</t>
-        </is>
-      </c>
+      <c r="A15" s="7" t="n"/>
     </row>
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>★ Budget note: all components except the Logitech G29 were provided by the university or were already on hand. The team's out-of-pocket budget consisted solely of the G29 driving simulator ($249.99).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
+          <t>Budget note: all components except the Logitech G29 were already on hand. Our out-of-pocket budget consisted solely of the G29 driving simulator, shared amongst the other capstone teams.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A15:G15"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>